<commit_message>
Add multiplex activation channel to deck and cost workbook
Deck: four new slides (rationale, foyer concept, 14-multiplex network,
commercials) proposing PVR/INOX cinema-foyer activation in the same
malls, since long-term atrium rental space is limited. Now 16 slides.

Cost workbook: new "Cinema Activation" tab (14 PVR/INOX sites, Rs 3,00,000
per site / 6 weeks, +18% GST) and a Summary alternative-channel block
giving a multiplex-option grand total alongside the atrium option.
Vendor "Khushi Advertising" replaced with ProMarcom in all terms.
Em-dashes removed from the preview for house tone.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SPjFYHW1nTDVr5tUuToRXR
</commit_message>
<xml_diff>
--- a/doft_diwali_popup/Doft_Kiosk_Cost_Workbook.xlsx
+++ b/doft_diwali_popup/Doft_Kiosk_Cost_Workbook.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Cost" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manpower Cost" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location Charges" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Elements" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinema Activation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Elements" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="₹#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -136,6 +137,17 @@
       <color rgb="00A9813A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C6A24E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00D8CDB6"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -229,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -325,6 +337,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -384,6 +402,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -750,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1067,68 +1094,122 @@
       <c r="E21" s="32" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="33" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Alternative location channel  -  Multiplex activation</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>D2. Multiplex activation (14 PVR/INOX, 6 wk)</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Cinema Activation</t>
+        </is>
+      </c>
+      <c r="D24" s="14">
+        <f>'Cinema Activation'!H19</f>
+        <v/>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Alternative to atrium (D); ex-GST</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL  -  multiplex option (incl. fee &amp; GST)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="33">
+        <f>(D11+D12+D13+'Cinema Activation'!H19)*(1+$C$7)*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="E25" s="34" t="inlineStr">
+        <is>
+          <t>A + B + C + multiplex, then fee &amp; GST</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
         <is>
           <t>Basis &amp; notes:</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="34" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="36" t="inlineStr">
         <is>
           <t>- Figures sourced from the execution-agency ops sheet (build + manpower + logistics + insurance) and the mall activation rate card.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="34" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="36" t="inlineStr">
         <is>
           <t>- Location / mall space (D) is a 3-day (Fri-Sun) rate card, ex-GST; the 6-week festive licence, CAM, electricity and deposits are to be negotiated per mall (blank).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="34" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>- Management fee modelled at 10% of programme sub-total (the source sheet contained an apparent calculation error on this line).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="34" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>- Billing hardware/software and security deposits left blank pending confirmation.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="34" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>- All rates indicative placeholders; confirm against vendor, mall and statutory quotes before commercial submission.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="22">
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="E14:F14"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="E19:F19"/>
-    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="E13:F13"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E25:F25"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E18:F18"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1152,14 +1233,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Cities &amp; Malls  -  Revised List (14)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>Per the client's revised preferred-mall list. Footfall &amp; activity location per the mall rate card.</t>
         </is>
@@ -1198,7 +1279,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="38" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -1211,54 +1292,54 @@
           <t>Select Citywalk</t>
         </is>
       </c>
-      <c r="D5" s="37" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>Saket</t>
         </is>
       </c>
-      <c r="E5" s="36" t="inlineStr">
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="F5" s="36" t="inlineStr">
+      <c r="F5" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="n">
+      <c r="A6" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>Noida</t>
         </is>
       </c>
-      <c r="C6" s="40" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>DLF Mall of India</t>
         </is>
       </c>
-      <c r="D6" s="41" t="inlineStr">
+      <c r="D6" s="43" t="inlineStr">
         <is>
           <t>Noida</t>
         </is>
       </c>
-      <c r="E6" s="38" t="inlineStr">
+      <c r="E6" s="40" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="F6" s="38" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n">
+      <c r="A7" s="38" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -1271,54 +1352,54 @@
           <t>Ambience Mall</t>
         </is>
       </c>
-      <c r="D7" s="37" t="inlineStr">
+      <c r="D7" s="39" t="inlineStr">
         <is>
           <t>Gurgaon</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="F7" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="38" t="n">
+      <c r="A8" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>Chandigarh</t>
         </is>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>Elante Mall</t>
         </is>
       </c>
-      <c r="D8" s="41" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>Industrial Area</t>
         </is>
       </c>
-      <c r="E8" s="38" t="inlineStr">
+      <c r="E8" s="40" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="F8" s="38" t="inlineStr">
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n">
+      <c r="A9" s="38" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -1331,54 +1412,54 @@
           <t>Lulu Mall</t>
         </is>
       </c>
-      <c r="D9" s="37" t="inlineStr">
+      <c r="D9" s="39" t="inlineStr">
         <is>
           <t>Hariharpur</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="38" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="F9" s="36" t="inlineStr">
+      <c r="F9" s="38" t="inlineStr">
         <is>
           <t>40-45k</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="38" t="n">
+      <c r="A10" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="39" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>Mumbai (BKC)</t>
         </is>
       </c>
-      <c r="C10" s="40" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Jio World Mall</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>BKC</t>
         </is>
       </c>
-      <c r="E10" s="38" t="inlineStr">
+      <c r="E10" s="40" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="F10" s="38" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="n">
+      <c r="A11" s="38" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -1391,54 +1472,54 @@
           <t>Phoenix Palladium</t>
         </is>
       </c>
-      <c r="D11" s="37" t="inlineStr">
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>Lower Parel</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" s="38" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="F11" s="36" t="inlineStr">
+      <c r="F11" s="38" t="inlineStr">
         <is>
           <t>40-45k</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="38" t="n">
+      <c r="A12" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="39" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>Ahmedabad</t>
         </is>
       </c>
-      <c r="C12" s="40" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>Phoenix / Palladium</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Thaltej</t>
         </is>
       </c>
-      <c r="E12" s="38" t="inlineStr">
+      <c r="E12" s="40" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="F12" s="38" t="inlineStr">
+      <c r="F12" s="40" t="inlineStr">
         <is>
           <t>40-45k</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="n">
+      <c r="A13" s="38" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -1451,54 +1532,54 @@
           <t>VR Mall</t>
         </is>
       </c>
-      <c r="D13" s="37" t="inlineStr">
+      <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Untkhana</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="E13" s="38" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="F13" s="36" t="inlineStr">
+      <c r="F13" s="38" t="inlineStr">
         <is>
           <t>30-35k</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="n">
+      <c r="A14" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="39" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
         <is>
           <t>Kolkata</t>
         </is>
       </c>
-      <c r="C14" s="40" t="inlineStr">
+      <c r="C14" s="42" t="inlineStr">
         <is>
           <t>South City Mall</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Jadavpur</t>
         </is>
       </c>
-      <c r="E14" s="38" t="inlineStr">
+      <c r="E14" s="40" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="F14" s="38" t="inlineStr">
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="n">
+      <c r="A15" s="38" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -1511,54 +1592,54 @@
           <t>Phoenix Marketcity</t>
         </is>
       </c>
-      <c r="D15" s="37" t="inlineStr">
+      <c r="D15" s="39" t="inlineStr">
         <is>
           <t>Velachery</t>
         </is>
       </c>
-      <c r="E15" s="36" t="inlineStr">
+      <c r="E15" s="38" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="F15" s="36" t="inlineStr">
+      <c r="F15" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="n">
+      <c r="A16" s="40" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="39" t="inlineStr">
+      <c r="B16" s="41" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="C16" s="40" t="inlineStr">
+      <c r="C16" s="42" t="inlineStr">
         <is>
           <t>Phoenix Marketcity</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Whitefield</t>
         </is>
       </c>
-      <c r="E16" s="38" t="inlineStr">
+      <c r="E16" s="40" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="F16" s="38" t="inlineStr">
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="36" t="n">
+      <c r="A17" s="38" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -1571,47 +1652,47 @@
           <t>Phoenix / Sarath City</t>
         </is>
       </c>
-      <c r="D17" s="37" t="inlineStr">
+      <c r="D17" s="39" t="inlineStr">
         <is>
           <t>Gachibowli</t>
         </is>
       </c>
-      <c r="E17" s="36" t="inlineStr">
+      <c r="E17" s="38" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="F17" s="36" t="inlineStr">
+      <c r="F17" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="n">
+      <c r="A18" s="40" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="39" t="inlineStr">
+      <c r="B18" s="41" t="inlineStr">
         <is>
           <t>Kochi</t>
         </is>
       </c>
-      <c r="C18" s="40" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
         <is>
           <t>Lulu International Mall</t>
         </is>
       </c>
-      <c r="D18" s="41" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Ernakulam</t>
         </is>
       </c>
-      <c r="E18" s="38" t="inlineStr">
+      <c r="E18" s="40" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="F18" s="38" t="inlineStr">
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
@@ -1626,7 +1707,7 @@
       </c>
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="n"/>
-      <c r="E19" s="42">
+      <c r="E19" s="44">
         <f>COUNTA(B5:B18)</f>
         <v/>
       </c>
@@ -1660,14 +1741,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Setup Cost  -  Kiosk Design, Build &amp; Install</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>8 ft x 8 ft kiosk. Headline build cost per execution-agency quote (Rs 3,50,000/kiosk); component split below is indicative.</t>
         </is>
@@ -1711,7 +1792,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="38" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -1719,20 +1800,20 @@
           <t>Structure &amp; framework</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
+      <c r="C5" s="45" t="inlineStr">
         <is>
           <t>MS/GI frame, base platform, carcass</t>
         </is>
       </c>
-      <c r="D5" s="36" t="inlineStr">
+      <c r="D5" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E5" s="36" t="n">
+      <c r="E5" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="44" t="n">
+      <c r="F5" s="46" t="n">
         <v>55000</v>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -1742,7 +1823,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="n">
+      <c r="A6" s="38" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -1750,20 +1831,20 @@
           <t>Body cladding &amp; finish</t>
         </is>
       </c>
-      <c r="C6" s="43" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>Warm-white PU-lacquer panels, fluted detailing</t>
         </is>
       </c>
-      <c r="D6" s="36" t="inlineStr">
+      <c r="D6" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E6" s="36" t="n">
+      <c r="E6" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="44" t="n">
+      <c r="F6" s="46" t="n">
         <v>60000</v>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -1773,7 +1854,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n">
+      <c r="A7" s="38" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -1781,20 +1862,20 @@
           <t>Counters</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="45" t="inlineStr">
         <is>
           <t>Black-stone tops, lockable storage bodies</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr">
+      <c r="D7" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E7" s="36" t="n">
+      <c r="E7" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="44" t="n">
+      <c r="F7" s="46" t="n">
         <v>45000</v>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -1804,7 +1885,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="n">
+      <c r="A8" s="38" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -1812,20 +1893,20 @@
           <t>Brass gallery shelving &amp; display</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>Backlit floating shelves, brass fronts</t>
         </is>
       </c>
-      <c r="D8" s="36" t="inlineStr">
+      <c r="D8" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E8" s="36" t="n">
+      <c r="E8" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="44" t="n">
+      <c r="F8" s="46" t="n">
         <v>45000</v>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -1835,7 +1916,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n">
+      <c r="A9" s="38" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -1843,20 +1924,20 @@
           <t>Backlit brand signage</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="45" t="inlineStr">
         <is>
           <t>Illuminated seal wall, fascia, backlit counter fronts</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
+      <c r="D9" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E9" s="36" t="n">
+      <c r="E9" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="44" t="n">
+      <c r="F9" s="46" t="n">
         <v>40000</v>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -1866,7 +1947,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="n">
+      <c r="A10" s="38" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -1874,20 +1955,20 @@
           <t>Lighting</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>Warm LED strips, drivers, downlights</t>
         </is>
       </c>
-      <c r="D10" s="36" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E10" s="36" t="n">
+      <c r="E10" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="44" t="n">
+      <c r="F10" s="46" t="n">
         <v>25000</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
@@ -1897,7 +1978,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="n">
+      <c r="A11" s="38" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -1905,20 +1986,20 @@
           <t>Electrical</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>Concealed wiring, DB/MCB, sockets</t>
         </is>
       </c>
-      <c r="D11" s="36" t="inlineStr">
+      <c r="D11" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="E11" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="44" t="n">
+      <c r="F11" s="46" t="n">
         <v>15000</v>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -1928,7 +2009,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="n">
+      <c r="A12" s="38" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -1936,26 +2017,26 @@
           <t>Flooring &amp; platform</t>
         </is>
       </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>Deck finish, warm-LED perimeter</t>
         </is>
       </c>
-      <c r="D12" s="36" t="inlineStr">
+      <c r="D12" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E12" s="36" t="n">
+      <c r="E12" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="44" t="n">
+      <c r="F12" s="46" t="n">
         <v>18000</v>
       </c>
       <c r="G12" s="15" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="n">
+      <c r="A13" s="38" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -1963,26 +2044,26 @@
           <t>Digital brand screen + stand</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>Screen for brand film / catalogue</t>
         </is>
       </c>
-      <c r="D13" s="36" t="inlineStr">
+      <c r="D13" s="38" t="inlineStr">
         <is>
           <t>Nos</t>
         </is>
       </c>
-      <c r="E13" s="36" t="n">
+      <c r="E13" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="44" t="n">
+      <c r="F13" s="46" t="n">
         <v>12000</v>
       </c>
       <c r="G13" s="15" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="n">
+      <c r="A14" s="38" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -1990,26 +2071,26 @@
           <t>Furniture</t>
         </is>
       </c>
-      <c r="C14" s="43" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>Consultation table + 4 chairs</t>
         </is>
       </c>
-      <c r="D14" s="36" t="inlineStr">
+      <c r="D14" s="38" t="inlineStr">
         <is>
           <t>Set</t>
         </is>
       </c>
-      <c r="E14" s="36" t="n">
+      <c r="E14" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="44" t="n">
+      <c r="F14" s="46" t="n">
         <v>15000</v>
       </c>
       <c r="G14" s="15" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="n">
+      <c r="A15" s="38" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2017,26 +2098,26 @@
           <t>Graphics, styling &amp; props</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="45" t="inlineStr">
         <is>
           <t>Vinyls, Diwali dressing</t>
         </is>
       </c>
-      <c r="D15" s="36" t="inlineStr">
+      <c r="D15" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E15" s="36" t="n">
+      <c r="E15" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="44" t="n">
+      <c r="F15" s="46" t="n">
         <v>8000</v>
       </c>
       <c r="G15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="n">
+      <c r="A16" s="38" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2044,20 +2125,20 @@
           <t>Transport, install &amp; dismantle</t>
         </is>
       </c>
-      <c r="C16" s="43" t="inlineStr">
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>Delivery, on-site setup, dismantle</t>
         </is>
       </c>
-      <c r="D16" s="36" t="inlineStr">
+      <c r="D16" s="38" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="E16" s="36" t="n">
+      <c r="E16" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="44" t="n">
+      <c r="F16" s="46" t="n">
         <v>12000</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
@@ -2076,7 +2157,7 @@
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
-      <c r="F17" s="45">
+      <c r="F17" s="47">
         <f>SUM(F5:F16)</f>
         <v/>
       </c>
@@ -2084,18 +2165,18 @@
     </row>
     <row r="18">
       <c r="A18" s="29" t="n"/>
-      <c r="B18" s="46" t="inlineStr">
+      <c r="B18" s="48" t="inlineStr">
         <is>
           <t>Programme setup (x 14 kiosks)</t>
         </is>
       </c>
       <c r="C18" s="29" t="n"/>
       <c r="D18" s="29" t="n"/>
-      <c r="E18" s="47">
+      <c r="E18" s="49">
         <f>Summary!$C$4</f>
         <v/>
       </c>
-      <c r="F18" s="48">
+      <c r="F18" s="50">
         <f>F17*Summary!$C$4</f>
         <v/>
       </c>
@@ -2130,14 +2211,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Manpower Cost</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>Per-kiosk deployment for the operating window; city-level roles added per city. Rates per execution-agency sheet.</t>
         </is>
@@ -2186,7 +2267,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="38" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -2194,18 +2275,18 @@
           <t>Sales Executive</t>
         </is>
       </c>
-      <c r="C5" s="36" t="inlineStr">
+      <c r="C5" s="38" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="D5" s="49" t="n">
+      <c r="D5" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="44" t="n">
+      <c r="E5" s="46" t="n">
         <v>1600</v>
       </c>
-      <c r="F5" s="49" t="n">
+      <c r="F5" s="51" t="n">
         <v>45</v>
       </c>
       <c r="G5" s="14">
@@ -2219,7 +2300,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="n">
+      <c r="A6" s="38" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -2227,18 +2308,18 @@
           <t>Helper</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="D6" s="49" t="n">
+      <c r="D6" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="44" t="n">
+      <c r="E6" s="46" t="n">
         <v>1200</v>
       </c>
-      <c r="F6" s="49" t="n">
+      <c r="F6" s="51" t="n">
         <v>42</v>
       </c>
       <c r="G6" s="14">
@@ -2252,7 +2333,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n">
+      <c r="A7" s="38" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2260,18 +2341,18 @@
           <t>Supervisor</t>
         </is>
       </c>
-      <c r="C7" s="36" t="inlineStr">
+      <c r="C7" s="38" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="D7" s="49" t="n">
+      <c r="D7" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="44" t="n">
+      <c r="E7" s="46" t="n">
         <v>1800</v>
       </c>
-      <c r="F7" s="49" t="n">
+      <c r="F7" s="51" t="n">
         <v>42</v>
       </c>
       <c r="G7" s="14">
@@ -2285,7 +2366,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="n">
+      <c r="A8" s="38" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -2293,18 +2374,18 @@
           <t>Training Support</t>
         </is>
       </c>
-      <c r="C8" s="36" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Lump</t>
         </is>
       </c>
-      <c r="D8" s="49" t="n">
+      <c r="D8" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="44" t="n">
+      <c r="E8" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="F8" s="49" t="n">
+      <c r="F8" s="51" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="14">
@@ -2318,7 +2399,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n">
+      <c r="A9" s="38" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2326,18 +2407,18 @@
           <t>Store Operations &amp; Cash</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
+      <c r="C9" s="38" t="inlineStr">
         <is>
           <t>Lump</t>
         </is>
       </c>
-      <c r="D9" s="49" t="n">
+      <c r="D9" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="44" t="n">
+      <c r="E9" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="F9" s="49" t="n">
+      <c r="F9" s="51" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="14">
@@ -2351,7 +2432,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="n">
+      <c r="A10" s="38" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -2359,18 +2440,18 @@
           <t>Reporting</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="D10" s="49" t="n">
+      <c r="D10" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="44" t="n">
+      <c r="E10" s="46" t="n">
         <v>150</v>
       </c>
-      <c r="F10" s="49" t="n">
+      <c r="F10" s="51" t="n">
         <v>45</v>
       </c>
       <c r="G10" s="14">
@@ -2415,7 +2496,7 @@
       <c r="H13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="n">
+      <c r="A14" s="38" t="n">
         <v>1</v>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2423,18 +2504,18 @@
           <t>City Manager</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="D14" s="49" t="n">
+      <c r="D14" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="44" t="n">
+      <c r="E14" s="46" t="n">
         <v>50000</v>
       </c>
-      <c r="F14" s="49" t="n">
+      <c r="F14" s="51" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="14">
@@ -2448,7 +2529,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="n">
+      <c r="A15" s="38" t="n">
         <v>2</v>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2456,18 +2537,18 @@
           <t>Trained Backup Bench</t>
         </is>
       </c>
-      <c r="C15" s="36" t="inlineStr">
+      <c r="C15" s="38" t="inlineStr">
         <is>
           <t>Lump</t>
         </is>
       </c>
-      <c r="D15" s="49" t="n">
+      <c r="D15" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="44" t="n">
+      <c r="E15" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="F15" s="49" t="n">
+      <c r="F15" s="51" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="14">
@@ -2499,7 +2580,7 @@
     </row>
     <row r="17">
       <c r="A17" s="29" t="n"/>
-      <c r="B17" s="46" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>Programme manpower  (per-kiosk + per-city) x 14</t>
         </is>
@@ -2508,7 +2589,7 @@
       <c r="D17" s="29" t="n"/>
       <c r="E17" s="29" t="n"/>
       <c r="F17" s="29" t="n"/>
-      <c r="G17" s="48">
+      <c r="G17" s="50">
         <f>(G11+G16)*Summary!$C$4</f>
         <v/>
       </c>
@@ -2544,68 +2625,68 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Location Charges  -  Mall Space</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>Mall activation rate card (3-day Fri-Sun, ex-GST). 6-week festive licence to be negotiated (left blank). GST 18% extra.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="52" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="51" t="inlineStr">
+      <c r="B4" s="53" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="C4" s="51" t="inlineStr">
+      <c r="C4" s="53" t="inlineStr">
         <is>
           <t>Mall</t>
         </is>
       </c>
-      <c r="D4" s="51" t="inlineStr">
+      <c r="D4" s="53" t="inlineStr">
         <is>
           <t>Activity Location</t>
         </is>
       </c>
-      <c r="E4" s="51" t="inlineStr">
+      <c r="E4" s="53" t="inlineStr">
         <is>
           <t>Weekend Footfall</t>
         </is>
       </c>
-      <c r="F4" s="50" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="G4" s="50" t="inlineStr">
+      <c r="G4" s="52" t="inlineStr">
         <is>
           <t>3-day rate (Rs, ex-GST)</t>
         </is>
       </c>
-      <c r="H4" s="50" t="inlineStr">
+      <c r="H4" s="52" t="inlineStr">
         <is>
           <t>6-wk licence (Rs)</t>
         </is>
       </c>
-      <c r="I4" s="51" t="inlineStr">
+      <c r="I4" s="53" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="38" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -2613,30 +2694,30 @@
           <t>Delhi NCR</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="54" t="inlineStr">
         <is>
           <t>Select City Walk</t>
         </is>
       </c>
-      <c r="D5" s="37" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>Mac Atrium</t>
         </is>
       </c>
-      <c r="E5" s="36" t="inlineStr">
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F5" s="36" t="inlineStr">
+      <c r="F5" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G5" s="44" t="n">
+      <c r="G5" s="46" t="n">
         <v>840000</v>
       </c>
-      <c r="H5" s="44" t="n"/>
+      <c r="H5" s="46" t="n"/>
       <c r="I5" s="15" t="inlineStr">
         <is>
           <t>Incl. Police &amp; MCD permission</t>
@@ -2644,7 +2725,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="n">
+      <c r="A6" s="38" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -2652,30 +2733,30 @@
           <t>Noida</t>
         </is>
       </c>
-      <c r="C6" s="52" t="inlineStr">
+      <c r="C6" s="54" t="inlineStr">
         <is>
           <t>DLF Mall of India</t>
         </is>
       </c>
-      <c r="D6" s="37" t="inlineStr">
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>Main Atrium</t>
         </is>
       </c>
-      <c r="E6" s="36" t="inlineStr">
+      <c r="E6" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F6" s="36" t="inlineStr">
+      <c r="F6" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G6" s="44" t="n">
+      <c r="G6" s="46" t="n">
         <v>728000</v>
       </c>
-      <c r="H6" s="44" t="n"/>
+      <c r="H6" s="46" t="n"/>
       <c r="I6" s="15" t="inlineStr">
         <is>
           <t>DLF do's &amp; don'ts apply</t>
@@ -2683,7 +2764,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n">
+      <c r="A7" s="38" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2691,30 +2772,30 @@
           <t>Gurgaon</t>
         </is>
       </c>
-      <c r="C7" s="52" t="inlineStr">
+      <c r="C7" s="54" t="inlineStr">
         <is>
           <t>Ambience Mall</t>
         </is>
       </c>
-      <c r="D7" s="37" t="inlineStr">
+      <c r="D7" s="39" t="inlineStr">
         <is>
           <t>Uniqlo Atrium</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="F7" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G7" s="44" t="n">
+      <c r="G7" s="46" t="n">
         <v>840000</v>
       </c>
-      <c r="H7" s="44" t="n"/>
+      <c r="H7" s="46" t="n"/>
       <c r="I7" s="15" t="inlineStr">
         <is>
           <t>Incl. Police &amp; MCG permission</t>
@@ -2722,7 +2803,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="n">
+      <c r="A8" s="38" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -2730,34 +2811,34 @@
           <t>Chandigarh</t>
         </is>
       </c>
-      <c r="C8" s="52" t="inlineStr">
+      <c r="C8" s="54" t="inlineStr">
         <is>
           <t>Elante Mall</t>
         </is>
       </c>
-      <c r="D8" s="37" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>Atrium</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="E8" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="F8" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G8" s="44" t="n">
+      <c r="G8" s="46" t="n">
         <v>728000</v>
       </c>
-      <c r="H8" s="44" t="n"/>
+      <c r="H8" s="46" t="n"/>
       <c r="I8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n">
+      <c r="A9" s="38" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2765,34 +2846,34 @@
           <t>Lucknow</t>
         </is>
       </c>
-      <c r="C9" s="52" t="inlineStr">
+      <c r="C9" s="54" t="inlineStr">
         <is>
           <t>Lulu Mall</t>
         </is>
       </c>
-      <c r="D9" s="37" t="inlineStr">
+      <c r="D9" s="39" t="inlineStr">
         <is>
           <t>Atrium</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="38" t="inlineStr">
         <is>
           <t>40-45k</t>
         </is>
       </c>
-      <c r="F9" s="36" t="inlineStr">
+      <c r="F9" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G9" s="44" t="n">
+      <c r="G9" s="46" t="n">
         <v>532000</v>
       </c>
-      <c r="H9" s="44" t="n"/>
+      <c r="H9" s="46" t="n"/>
       <c r="I9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="n">
+      <c r="A10" s="38" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -2800,30 +2881,30 @@
           <t>Mumbai (BKC)</t>
         </is>
       </c>
-      <c r="C10" s="52" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
         <is>
           <t>Jio World Drive</t>
         </is>
       </c>
-      <c r="D10" s="37" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>GF Atrium</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F10" s="36" t="inlineStr">
+      <c r="F10" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G10" s="44" t="n">
+      <c r="G10" s="46" t="n">
         <v>784000</v>
       </c>
-      <c r="H10" s="44" t="n"/>
+      <c r="H10" s="46" t="n"/>
       <c r="I10" s="15" t="inlineStr">
         <is>
           <t>Incl. Police &amp; BMC permission</t>
@@ -2831,7 +2912,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="n">
+      <c r="A11" s="38" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -2839,30 +2920,30 @@
           <t>Mumbai (Lower Parel)</t>
         </is>
       </c>
-      <c r="C11" s="52" t="inlineStr">
+      <c r="C11" s="54" t="inlineStr">
         <is>
           <t>Phoenix Palladium</t>
         </is>
       </c>
-      <c r="D11" s="37" t="inlineStr">
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>Courtyard (open)</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" s="38" t="inlineStr">
         <is>
           <t>40-45k</t>
         </is>
       </c>
-      <c r="F11" s="36" t="inlineStr">
+      <c r="F11" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G11" s="44" t="n">
+      <c r="G11" s="46" t="n">
         <v>840000</v>
       </c>
-      <c r="H11" s="44" t="n"/>
+      <c r="H11" s="46" t="n"/>
       <c r="I11" s="15" t="inlineStr">
         <is>
           <t>Incl. Police &amp; BMC permission</t>
@@ -2870,7 +2951,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="n">
+      <c r="A12" s="38" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -2878,34 +2959,34 @@
           <t>Ahmedabad</t>
         </is>
       </c>
-      <c r="C12" s="52" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>Palladium Ahmedabad</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
+      <c r="D12" s="39" t="inlineStr">
         <is>
           <t>Atrium</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="E12" s="38" t="inlineStr">
         <is>
           <t>40-45k</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
+      <c r="F12" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G12" s="44" t="n">
+      <c r="G12" s="46" t="n">
         <v>784000</v>
       </c>
-      <c r="H12" s="44" t="n"/>
+      <c r="H12" s="46" t="n"/>
       <c r="I12" s="15" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="n">
+      <c r="A13" s="38" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2913,34 +2994,34 @@
           <t>Nagpur</t>
         </is>
       </c>
-      <c r="C13" s="52" t="inlineStr">
+      <c r="C13" s="54" t="inlineStr">
         <is>
           <t>VR Mall</t>
         </is>
       </c>
-      <c r="D13" s="37" t="inlineStr">
+      <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Atrium</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="E13" s="38" t="inlineStr">
         <is>
           <t>30-35k</t>
         </is>
       </c>
-      <c r="F13" s="36" t="inlineStr">
+      <c r="F13" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G13" s="44" t="n">
+      <c r="G13" s="46" t="n">
         <v>308000</v>
       </c>
-      <c r="H13" s="44" t="n"/>
+      <c r="H13" s="46" t="n"/>
       <c r="I13" s="15" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="n">
+      <c r="A14" s="38" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2948,34 +3029,34 @@
           <t>Kolkata</t>
         </is>
       </c>
-      <c r="C14" s="52" t="inlineStr">
+      <c r="C14" s="54" t="inlineStr">
         <is>
           <t>South City Mall</t>
         </is>
       </c>
-      <c r="D14" s="37" t="inlineStr">
+      <c r="D14" s="39" t="inlineStr">
         <is>
           <t>Main Atrium</t>
         </is>
       </c>
-      <c r="E14" s="36" t="inlineStr">
+      <c r="E14" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F14" s="36" t="inlineStr">
+      <c r="F14" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G14" s="44" t="n">
+      <c r="G14" s="46" t="n">
         <v>336000</v>
       </c>
-      <c r="H14" s="44" t="n"/>
+      <c r="H14" s="46" t="n"/>
       <c r="I14" s="15" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="n">
+      <c r="A15" s="38" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2983,34 +3064,34 @@
           <t>Chennai</t>
         </is>
       </c>
-      <c r="C15" s="52" t="inlineStr">
+      <c r="C15" s="54" t="inlineStr">
         <is>
           <t>Phoenix Market City</t>
         </is>
       </c>
-      <c r="D15" s="37" t="inlineStr">
+      <c r="D15" s="39" t="inlineStr">
         <is>
           <t>Atrium</t>
         </is>
       </c>
-      <c r="E15" s="36" t="inlineStr">
+      <c r="E15" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F15" s="36" t="inlineStr">
+      <c r="F15" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G15" s="44" t="n">
+      <c r="G15" s="46" t="n">
         <v>700000</v>
       </c>
-      <c r="H15" s="44" t="n"/>
+      <c r="H15" s="46" t="n"/>
       <c r="I15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="n">
+      <c r="A16" s="38" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -3018,34 +3099,34 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="C16" s="52" t="inlineStr">
+      <c r="C16" s="54" t="inlineStr">
         <is>
           <t>Phoenix Market City</t>
         </is>
       </c>
-      <c r="D16" s="37" t="inlineStr">
+      <c r="D16" s="39" t="inlineStr">
         <is>
           <t>Main Atrium</t>
         </is>
       </c>
-      <c r="E16" s="36" t="inlineStr">
+      <c r="E16" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F16" s="36" t="inlineStr">
+      <c r="F16" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G16" s="44" t="n">
+      <c r="G16" s="46" t="n">
         <v>560000</v>
       </c>
-      <c r="H16" s="44" t="n"/>
+      <c r="H16" s="46" t="n"/>
       <c r="I16" s="15" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="36" t="n">
+      <c r="A17" s="38" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -3053,30 +3134,30 @@
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="C17" s="52" t="inlineStr">
+      <c r="C17" s="54" t="inlineStr">
         <is>
           <t>Sarath City Capital</t>
         </is>
       </c>
-      <c r="D17" s="37" t="inlineStr">
+      <c r="D17" s="39" t="inlineStr">
         <is>
           <t>Main Atrium</t>
         </is>
       </c>
-      <c r="E17" s="36" t="inlineStr">
+      <c r="E17" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F17" s="36" t="inlineStr">
+      <c r="F17" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G17" s="44" t="n">
+      <c r="G17" s="46" t="n">
         <v>532000</v>
       </c>
-      <c r="H17" s="44" t="n"/>
+      <c r="H17" s="46" t="n"/>
       <c r="I17" s="15" t="inlineStr">
         <is>
           <t>Inorbit alt: Rs 5,60,000</t>
@@ -3084,7 +3165,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="36" t="n">
+      <c r="A18" s="38" t="n">
         <v>14</v>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -3092,30 +3173,30 @@
           <t>Kochi</t>
         </is>
       </c>
-      <c r="C18" s="52" t="inlineStr">
+      <c r="C18" s="54" t="inlineStr">
         <is>
           <t>Lulu International Mall</t>
         </is>
       </c>
-      <c r="D18" s="37" t="inlineStr">
+      <c r="D18" s="39" t="inlineStr">
         <is>
           <t>Main Atrium</t>
         </is>
       </c>
-      <c r="E18" s="36" t="inlineStr">
+      <c r="E18" s="38" t="inlineStr">
         <is>
           <t>50-60k</t>
         </is>
       </c>
-      <c r="F18" s="36" t="inlineStr">
+      <c r="F18" s="38" t="inlineStr">
         <is>
           <t>8x8ft</t>
         </is>
       </c>
-      <c r="G18" s="44" t="n">
+      <c r="G18" s="46" t="n">
         <v>840000</v>
       </c>
-      <c r="H18" s="44" t="n"/>
+      <c r="H18" s="46" t="n"/>
       <c r="I18" s="15" t="inlineStr"/>
     </row>
     <row r="19">
@@ -3129,7 +3210,7 @@
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="8" t="n"/>
-      <c r="G19" s="45">
+      <c r="G19" s="47">
         <f>SUM(G5:G18)</f>
         <v/>
       </c>
@@ -3137,28 +3218,28 @@
       <c r="I19" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="33" t="inlineStr">
+      <c r="A21" s="35" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="34" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>- Rates are 3-day (Fri-Sun) activation rates, ex-GST, per the mall rate card; non-festive - festive rates may vary.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="34" t="inlineStr">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>- 6-week festive-season licence, CAM, electricity above 3-4 KVA and security deposits to be negotiated per mall (left blank).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="34" t="inlineStr">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>- Booking against 100% advance; rates valid 15 days; PPL/IPRS and special permissions extra.</t>
         </is>
@@ -3183,6 +3264,663 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>Cinema / Multiplex Activation  -  Alternative Location</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>8x8 ft foyer activation in the PVR / INOX multiplexes at the same malls. 6-week cost per site; GST 18% extra. Managed by ProMarcom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="53" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C4" s="53" t="inlineStr">
+        <is>
+          <t>Multiplex / Cinema</t>
+        </is>
+      </c>
+      <c r="D4" s="53" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Seats / show</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Space</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="inlineStr">
+        <is>
+          <t>Cost - 6 weeks (Rs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Mumbai (Lower Parel)</t>
+        </is>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>PVR Phoenix (Worli)</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="55" t="n">
+        <v>1275</v>
+      </c>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Mumbai (BKC)</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>PVR Maison BKC</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" s="55" t="n">
+        <v>882</v>
+      </c>
+      <c r="G6" s="38" t="inlineStr">
+        <is>
+          <t>6x6</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Ahmedabad</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>PVR Palladium</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E7" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="55" t="n">
+        <v>1283</v>
+      </c>
+      <c r="G7" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Delhi (Saket)</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>PVR Select Citywalk</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E8" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="55" t="n">
+        <v>1056</v>
+      </c>
+      <c r="G8" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>PVR DT - Mall of India</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="55" t="n">
+        <v>1712</v>
+      </c>
+      <c r="G9" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Gurgaon</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>PVR Ambience Mall</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="n">
+        <v>11</v>
+      </c>
+      <c r="F10" s="55" t="n">
+        <v>1122</v>
+      </c>
+      <c r="G10" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H10" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Chandigarh</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>PVR Nexus Elante</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="55" t="n">
+        <v>1599</v>
+      </c>
+      <c r="G11" s="38" t="inlineStr">
+        <is>
+          <t>6x6</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>PVR Superplex - Lulu</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" s="55" t="n">
+        <v>1841</v>
+      </c>
+      <c r="G12" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>INOX City Centre</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>PVR INOX</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="55" t="n">
+        <v>1144</v>
+      </c>
+      <c r="G13" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>INOX City Centre II</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>PVR INOX</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="55" t="n">
+        <v>1190</v>
+      </c>
+      <c r="G14" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>PVR Icon - Hitech City</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="55" t="n">
+        <v>936</v>
+      </c>
+      <c r="G15" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>PVR Phoenix Market City</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" s="55" t="n">
+        <v>1401</v>
+      </c>
+      <c r="G16" s="38" t="inlineStr">
+        <is>
+          <t>6x6</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="38" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>INOX Luxe - Phoenix</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>PVR INOX</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="n">
+        <v>11</v>
+      </c>
+      <c r="F17" s="55" t="n">
+        <v>2688</v>
+      </c>
+      <c r="G17" s="38" t="inlineStr">
+        <is>
+          <t>6x6</t>
+        </is>
+      </c>
+      <c r="H17" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Cochin</t>
+        </is>
+      </c>
+      <c r="C18" s="54" t="inlineStr">
+        <is>
+          <t>PVR Lulu Mall</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>PVR</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="F18" s="55" t="n">
+        <v>1926</v>
+      </c>
+      <c r="G18" s="38" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="H18" s="46" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Total - 14 multiplexes (ex-GST)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="9">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="56">
+        <f>SUM(F5:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="47">
+        <f>SUM(H5:H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="n"/>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>GST @ 18%</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="24" t="n"/>
+      <c r="G20" s="24" t="n"/>
+      <c r="H20" s="57">
+        <f>H19*Summary!$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="n"/>
+      <c r="B21" s="29" t="n"/>
+      <c r="C21" s="48" t="inlineStr">
+        <is>
+          <t>Total incl. GST</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="29" t="n"/>
+      <c r="F21" s="29" t="n"/>
+      <c r="G21" s="29" t="n"/>
+      <c r="H21" s="50">
+        <f>H19+H20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="inlineStr">
+        <is>
+          <t>Terms (per the multiplex rate card, managed by ProMarcom):</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t>- 100% advance, in favour of ProMarcom.  18% Govt. service tax extra on the above rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>- Availability to be confirmed before booking; site once booked cannot be postponed or cancelled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>- Billing from date of booking / availability; rates subject to change without prior notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t>- Alternative to the mall-atrium location (see Location Charges); proposed as atrium space on long-term rental is limited.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A27:H27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3195,14 +3933,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Other Elements</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>Logistics, insurance, operations and pass-through items (per kiosk / season). Hardware &amp; software left blank pending confirmation.</t>
         </is>
@@ -3241,7 +3979,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="38" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -3249,15 +3987,15 @@
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
+      <c r="C5" s="45" t="inlineStr">
         <is>
           <t>Stock pickup (Ghaziabad WH), first fill, replenishment, return of unsold</t>
         </is>
       </c>
-      <c r="D5" s="44" t="n">
+      <c r="D5" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="E5" s="36" t="inlineStr">
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>Per season</t>
         </is>
@@ -3265,7 +4003,7 @@
       <c r="F5" s="15" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="n">
+      <c r="A6" s="38" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -3273,15 +4011,15 @@
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="C6" s="43" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>Seasonal storage / stockroom</t>
         </is>
       </c>
-      <c r="D6" s="44" t="n">
+      <c r="D6" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="E6" s="36" t="inlineStr">
+      <c r="E6" s="38" t="inlineStr">
         <is>
           <t>Per season</t>
         </is>
@@ -3289,7 +4027,7 @@
       <c r="F6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n">
+      <c r="A7" s="38" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -3297,15 +4035,15 @@
           <t>Insurance - Fire</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="45" t="inlineStr">
         <is>
           <t>Mall fire insurance</t>
         </is>
       </c>
-      <c r="D7" s="44" t="n">
+      <c r="D7" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>Per season</t>
         </is>
@@ -3313,7 +4051,7 @@
       <c r="F7" s="15" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="n">
+      <c r="A8" s="38" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -3321,15 +4059,15 @@
           <t>Insurance - Transport</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>Stock in transit</t>
         </is>
       </c>
-      <c r="D8" s="44" t="n">
+      <c r="D8" s="46" t="n">
         <v>12000</v>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="E8" s="38" t="inlineStr">
         <is>
           <t>Per season</t>
         </is>
@@ -3337,7 +4075,7 @@
       <c r="F8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n">
+      <c r="A9" s="38" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -3345,15 +4083,15 @@
           <t>Extended Trading</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="45" t="inlineStr">
         <is>
           <t>Extended ops in select cities (Christmas &amp; New Year)</t>
         </is>
       </c>
-      <c r="D9" s="44" t="n">
+      <c r="D9" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="38" t="inlineStr">
         <is>
           <t>Select only</t>
         </is>
@@ -3361,7 +4099,7 @@
       <c r="F9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="n">
+      <c r="A10" s="38" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -3369,15 +4107,15 @@
           <t>Dismantle &amp; Stock Return</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>Dismantling, fixture removal, unsold-stock return</t>
         </is>
       </c>
-      <c r="D10" s="44" t="n">
+      <c r="D10" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>Post-season</t>
         </is>
@@ -3385,7 +4123,7 @@
       <c r="F10" s="15" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="n">
+      <c r="A11" s="38" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -3393,15 +4131,15 @@
           <t>Final Reconciliation</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>Commercial reconciliation &amp; season review</t>
         </is>
       </c>
-      <c r="D11" s="44" t="n">
+      <c r="D11" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" s="38" t="inlineStr">
         <is>
           <t>Project close</t>
         </is>
@@ -3409,7 +4147,7 @@
       <c r="F11" s="15" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="n">
+      <c r="A12" s="38" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -3417,13 +4155,13 @@
           <t>Billing Hardware</t>
         </is>
       </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>EDC / card machine, thermal printer, tablet, stand</t>
         </is>
       </c>
-      <c r="D12" s="44" t="n"/>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="D12" s="46" t="n"/>
+      <c r="E12" s="38" t="inlineStr">
         <is>
           <t>Per kiosk</t>
         </is>
@@ -3435,7 +4173,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="n">
+      <c r="A13" s="38" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -3443,13 +4181,13 @@
           <t>Billing Software</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>POS / billing software licence</t>
         </is>
       </c>
-      <c r="D13" s="44" t="n"/>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="D13" s="46" t="n"/>
+      <c r="E13" s="38" t="inlineStr">
         <is>
           <t>Per kiosk</t>
         </is>
@@ -3461,7 +4199,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="n">
+      <c r="A14" s="38" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -3469,13 +4207,13 @@
           <t>Security Deposit (refundable)</t>
         </is>
       </c>
-      <c r="C14" s="43" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>Mall / statutory deposits</t>
         </is>
       </c>
-      <c r="D14" s="44" t="n"/>
-      <c r="E14" s="36" t="inlineStr">
+      <c r="D14" s="46" t="n"/>
+      <c r="E14" s="38" t="inlineStr">
         <is>
           <t>Per mall</t>
         </is>
@@ -3503,13 +4241,13 @@
     </row>
     <row r="16">
       <c r="A16" s="29" t="n"/>
-      <c r="B16" s="46" t="inlineStr">
+      <c r="B16" s="48" t="inlineStr">
         <is>
           <t>Programme other (x 14 kiosks)</t>
         </is>
       </c>
       <c r="C16" s="29" t="n"/>
-      <c r="D16" s="48">
+      <c r="D16" s="50">
         <f>D15*Summary!$C$4</f>
         <v/>
       </c>

</xml_diff>